<commit_message>
nuevo modelo de excel para la precarga de solps
</commit_message>
<xml_diff>
--- a/SustitucionMOA/Documentacion/TemplatePrecargaSolp.xlsx
+++ b/SustitucionMOA/Documentacion/TemplatePrecargaSolp.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\emartin\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFCC3D36-0C91-4B4D-B008-79915E518C20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26EC610D-35A6-4E88-BE83-C6DF1DE17D6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10110" yWindow="-12630" windowWidth="22430" windowHeight="11030" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1040" yWindow="-13360" windowWidth="22430" windowHeight="11030" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -28,6 +28,7 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author/>
+    <author>Eugenio Martin</author>
   </authors>
   <commentList>
     <comment ref="N1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
@@ -147,6 +148,54 @@
             <charset val="1"/>
           </rPr>
           <t>Para servicios refiere a la subposición, para materiales al material</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="S1" authorId="1" shapeId="0" xr:uid="{4A615EC0-5F49-47B5-B52F-D4F4417266E5}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Eugenio Martin:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+Solo para material no catalogado</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="T1" authorId="1" shapeId="0" xr:uid="{F38A6632-7E0F-4730-82EE-D2792808157A}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Eugenio Martin:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+Solo para material no catalogado</t>
         </r>
       </text>
     </comment>
@@ -155,7 +204,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
   <si>
     <t>Nro posición</t>
   </si>
@@ -218,13 +267,19 @@
   </si>
   <si>
     <t>Precio</t>
+  </si>
+  <si>
+    <t>Motivo</t>
+  </si>
+  <si>
+    <t>Modelo</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -244,6 +299,19 @@
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -725,7 +793,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R11"/>
+  <dimension ref="A1:T11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="14.140625" customWidth="1"/>
@@ -739,7 +807,7 @@
     <col min="20" max="20" width="13.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="45" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:20" ht="45" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -794,25 +862,31 @@
       <c r="R1" s="2" t="s">
         <v>16</v>
       </c>
+      <c r="S1" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="T1" s="3" t="s">
+        <v>22</v>
+      </c>
     </row>
-    <row r="2" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="5"/>
     </row>
-    <row r="3" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5"/>
     </row>
-    <row r="4" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5"/>
     </row>
-    <row r="5" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5"/>
     </row>
-    <row r="6" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="5"/>
     </row>
-    <row r="7" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="8" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="11" spans="1:18" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="8" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="11" spans="1:20" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="L11" s="6" t="s">
         <v>17</v>
       </c>

</xml_diff>

<commit_message>
MOA-537 Se corrige el bug para servicios no catalogados que mostraba un numero Se corrige el bug que solo completa imputaciones de ceco Se agrega una nueva columna para completar el solicitante.
</commit_message>
<xml_diff>
--- a/SustitucionMOA/Documentacion/TemplatePrecargaSolp.xlsx
+++ b/SustitucionMOA/Documentacion/TemplatePrecargaSolp.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\emartin\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\emartin\source\repos\WebOperaciones\SustitucionMOA\Documentacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26EC610D-35A6-4E88-BE83-C6DF1DE17D6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93ECA71F-3C88-4529-B240-8BA4B3BE000D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1040" yWindow="-13360" windowWidth="22430" windowHeight="11030" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-14510" windowWidth="34620" windowHeight="13900" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -204,7 +204,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t>Nro posición</t>
   </si>
@@ -273,6 +273,9 @@
   </si>
   <si>
     <t>Modelo</t>
+  </si>
+  <si>
+    <t>Solicitante</t>
   </si>
 </sst>
 </file>
@@ -793,7 +796,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:T11"/>
+  <dimension ref="A1:U11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="14.140625" customWidth="1"/>
@@ -807,7 +810,7 @@
     <col min="20" max="20" width="13.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" ht="45" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:21" ht="45" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -868,25 +871,28 @@
       <c r="T1" s="3" t="s">
         <v>22</v>
       </c>
+      <c r="U1" s="2" t="s">
+        <v>23</v>
+      </c>
     </row>
-    <row r="2" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="5"/>
     </row>
-    <row r="3" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5"/>
     </row>
-    <row r="4" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5"/>
     </row>
-    <row r="5" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5"/>
     </row>
-    <row r="6" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="5"/>
     </row>
-    <row r="7" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="8" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="11" spans="1:20" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="8" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="11" spans="1:21" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="L11" s="6" t="s">
         <v>17</v>
       </c>

</xml_diff>